<commit_message>
Actualizacion INVIMA: Eliminacion de Listado de referencia, correccion en seleccion de Mezclas y actualizacion de plantilla
</commit_message>
<xml_diff>
--- a/plantilla_base.xlsx
+++ b/plantilla_base.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Grupos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Presentaciones comerciales" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Ingredientes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Fórmula Marco" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Composición por grupo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Características Organolépticas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grupos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Presentaciones comerciales" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ingredientes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fórmula Marco" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Composición por grupo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Características Organolépticas" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -619,25 +619,20 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Listado de referencia</t>
+          <t>Cantidad</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Cantidad</t>
+          <t>Unidad de medida</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Unidad de medida</t>
+          <t>¿Es nanomaterial?</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>¿Es nanomaterial?</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Tamaño de partícula (nm)</t>
         </is>
@@ -659,25 +654,20 @@
           <t>Humectante</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>CosIng</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="n">
+      <c r="D2" s="2" t="n">
         <v>5</v>
       </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -690,7 +680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -727,25 +717,20 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Listado de referencia</t>
+          <t>Cantidad</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Cantidad</t>
+          <t>Unidad de medida</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Unidad de medida</t>
+          <t>¿Es nanomaterial?</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>¿Es nanomaterial?</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Tamaño de partícula (nm)</t>
         </is>
@@ -772,25 +757,20 @@
           <t>Solvente</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>CosIng</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="n">
+      <c r="E2" s="2" t="n">
         <v>80</v>
       </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -803,7 +783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -846,25 +826,20 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Listado de referencia</t>
+          <t>Cantidad</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Cantidad</t>
+          <t>Unidad de medida</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Unidad de medida</t>
+          <t>¿Es nanomaterial?</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>¿Es nanomaterial?</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Tamaño de partícula (nm)</t>
         </is>
@@ -896,25 +871,20 @@
           <t>Colorante</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>CosIng</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="n">
+      <c r="F2" s="2" t="n">
         <v>2</v>
       </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>